<commit_message>
docs(permisos): aplicar H-2 — acceso de consulta del contratista al expediente (HU-04) fundamentado en art. 117 RLOPSRM, en matriz de permisos y de trazabilidad
</commit_message>
<xml_diff>
--- a/docs/Matriz_Permisos_SIGECOP.xlsx
+++ b/docs/Matriz_Permisos_SIGECOP.xlsx
@@ -1103,9 +1103,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -2191,12 +2191,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Residente, Supervisión, Dependencia</t>
+          <t>Residente, Supervisión, Dependencia, Contratista/Superint. (consulta)</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Art. 46 LOPSRM</t>
+          <t>Art. 46 LOPSRM; Art. 117 RLOPSRM (el superintendente debe conocer catálogo, programa, bitácora y documentos del contrato)</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs: actualizar columna Vista impl. de la matriz de permisos (todas las vistas construidas)
</commit_message>
<xml_diff>
--- a/docs/Matriz_Permisos_SIGECOP.xlsx
+++ b/docs/Matriz_Permisos_SIGECOP.xlsx
@@ -1073,7 +1073,7 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>